<commit_message>
feat: initial link products to GeneCopoeia publications
Implement corpus matching workflow that scans publication sentences for product aliases and associates matched articles with candidate GeneCopoeia products.
</commit_message>
<xml_diff>
--- a/data/genecopoeia_pipeline_test_raw_products/genecopoeia_pipeline_test_product_map.xlsx
+++ b/data/genecopoeia_pipeline_test_raw_products/genecopoeia_pipeline_test_product_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jingh\Projects\pub-proof\data\genecopoeia_pipeline_test_raw_products\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE89C2B-87E8-467C-98DC-968454E0CA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CDE084-B465-4665-8793-AE7E4ED44921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="213">
   <si>
     <t>LT001</t>
   </si>
@@ -42,18 +42,9 @@
     <t>BI001</t>
   </si>
   <si>
-    <t>LP341-100</t>
-  </si>
-  <si>
     <t>QP116</t>
   </si>
   <si>
-    <t>ER011</t>
-  </si>
-  <si>
-    <t>CC001</t>
-  </si>
-  <si>
     <t>Part ID</t>
   </si>
   <si>
@@ -378,9 +369,6 @@
     <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/BI001-scaled.jpg</t>
   </si>
   <si>
-    <t>https://www.genecopoeia.com//product/lentiviral-particles/</t>
-  </si>
-  <si>
     <t>Premade lentivirus</t>
   </si>
   <si>
@@ -399,30 +387,6 @@
     <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/QP1151-scaled.jpg</t>
   </si>
   <si>
-    <t>https://www.genecopoeia.com/product/cloning_products/ezshuttle-recombination-cloning-system/</t>
-  </si>
-  <si>
-    <t>Ezshuttle</t>
-  </si>
-  <si>
-    <t>https://www.genecopoeia.com/wp-content/uploads/2024/10/BP-II-Enzyme-Mix-US.pdf</t>
-  </si>
-  <si>
-    <t>https://www.genecopoeia.com/wp-content/uploads/2025/04/ER011-scaled.jpg</t>
-  </si>
-  <si>
-    <t>http://www.genecopoeia.com/product/competent-cells/</t>
-  </si>
-  <si>
-    <t>10 tubes</t>
-  </si>
-  <si>
-    <t>Comp cells</t>
-  </si>
-  <si>
-    <t>https://www.genecopoeia.com/wp-content/uploads/2025/08/CC001-US-scaled.jpg</t>
-  </si>
-  <si>
     <t>4–8°C (Stable for at least 6 months) Alternatively, the packaging mix can be stored at -80 °C in usable aliquots. Avoid repeated freezing/ thawing.</t>
   </si>
   <si>
@@ -441,9 +405,6 @@
     <t>(-80°C)</t>
   </si>
   <si>
-    <t>eGFP-Lv195 Lentifect™ Purified Lentiviral Particles (25 µl x 4 vial)(Old cat # LP319-100)</t>
-  </si>
-  <si>
     <t>25 µl x 4 vial</t>
   </si>
   <si>
@@ -453,13 +414,256 @@
     <t>–20°C (Stable for at least 12 months) Alternatively, the solution can also be stored at –80°C in aliquots. Avoid repeated freezing/ thawing.</t>
   </si>
   <si>
-    <t>EZRecombinase™ LR II Enzyme Mix (-20?)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">–20°C </t>
-  </si>
-  <si>
-    <t>GCI-5? Chemically Competent E.coli Cells, (10 tubes)</t>
+    <t>LT002</t>
+  </si>
+  <si>
+    <t>LF032</t>
+  </si>
+  <si>
+    <t>LF031</t>
+  </si>
+  <si>
+    <t>LF062</t>
+  </si>
+  <si>
+    <t>EF014</t>
+  </si>
+  <si>
+    <t>LT007</t>
+  </si>
+  <si>
+    <t>QP115</t>
+  </si>
+  <si>
+    <t>LF033</t>
+  </si>
+  <si>
+    <t>LF006</t>
+  </si>
+  <si>
+    <t>LF009</t>
+  </si>
+  <si>
+    <t>QP029</t>
+  </si>
+  <si>
+    <t>EF001</t>
+  </si>
+  <si>
+    <t>LP721-100</t>
+  </si>
+  <si>
+    <t>LP303-025</t>
+  </si>
+  <si>
+    <t>EF002</t>
+  </si>
+  <si>
+    <t>PA001-V2</t>
+  </si>
+  <si>
+    <t>Systemic Autoimmune-associated Antigen Array</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/autoantigen-general-survey/</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2019/11/Protein-array-website-Figure-1-v-3.jpg</t>
+  </si>
+  <si>
+    <t>Workflow for autoantibody profiling in samples using GeneCopoeia’s OmicsArray™ antigen microarrays.</t>
+  </si>
+  <si>
+    <t>120-plex</t>
+  </si>
+  <si>
+    <t>antigen array</t>
+  </si>
+  <si>
+    <t>120 superior-quality purifiedproteins and 8 controls</t>
+  </si>
+  <si>
+    <t>–20°C (Stable for at least 12 months)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2020/09/OmicsArray-Antigen-Microarray-User-Manual-20200909.pdf</t>
+  </si>
+  <si>
+    <t>Lenti-Pac HIV Expression Packaging Kit (40 reactions)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LT002%E6%96%B0-scaled.jpg</t>
+  </si>
+  <si>
+    <t>40 reactions</t>
+  </si>
+  <si>
+    <t>Secrete-Pair Dual Luminescence Assay Kit (300 rxns)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/dual-luminescence-assay/</t>
+  </si>
+  <si>
+    <t>300reactions</t>
+  </si>
+  <si>
+    <t>Luciferase kit</t>
+  </si>
+  <si>
+    <t>Ice pack</t>
+  </si>
+  <si>
+    <t>-20°C Stable at least 6 months</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2017/02/Secrete-Pair-%E2%84%A2-Luminescence-Assay-Kit-protocol-20160516.pdf</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF032-scaled.jpg</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2016/09/MSDS_secrete_pair-kits.pdf</t>
+  </si>
+  <si>
+    <t>Secrete-Pair Dual Luminescence Assay Kit (100 rxns)</t>
+  </si>
+  <si>
+    <t>100 reactions</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF031?1?-scaled.jpg</t>
+  </si>
+  <si>
+    <t>Secrete-Pair Gaussia Luciferase Assay Kit (1000 rxns)</t>
+  </si>
+  <si>
+    <t>1000 reactions</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF062-scaled.jpg</t>
+  </si>
+  <si>
+    <t>EndoFectin™ Max transfection reagent (3ml)</t>
+  </si>
+  <si>
+    <t>3ml</t>
+  </si>
+  <si>
+    <t>Lenti-Pac™ Lentivirus Concentration Solution (50 ml)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2025/08/LT007-US-scaled.jpg</t>
+  </si>
+  <si>
+    <t>50 ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4°C </t>
+  </si>
+  <si>
+    <t>All-in-One™ miRNA qRT-PCR Detection Kit 2.0* (20 RT and 200 qPCR reactions) (Old cat # QP015)</t>
+  </si>
+  <si>
+    <t>20 RT and 200 qPCR reactions</t>
+  </si>
+  <si>
+    <t>Secrete-Pair Dual Luminescence Assay Kit (1000 rxns)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF033-3-scaled.jpg</t>
+  </si>
+  <si>
+    <t>LP519-025</t>
+  </si>
+  <si>
+    <t>shRNA Scrambled Control-LVRU6GP Lentiviral Particles (25 µl x 1 vial) (Old cat # LPP-CSHCTR001-LVRU6GP-025-C)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/lentivirus-system/purified-lentiviral-particles/lentiviral-particles/</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2019/12/CSHCTR001-LVRU6GP-LP519-025-LP519-100.pdf</t>
+  </si>
+  <si>
+    <t>GeneCopoeia Premade lentivirus</t>
+  </si>
+  <si>
+    <t>25 µl x 1 vial</t>
+  </si>
+  <si>
+    <t>Luc-Pair Duo-Luciferase HS Assay Kits (1000rxns)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/luc-pair-duo-luciferase-hs-assay-kit/</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2017/02/Luc-Pair-%E2%84%A2-Duo-Luciferase-HS-Assay-Kit-protocol.pdf</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF006%E6%96%B0-scaled.jpg</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2016/12/MSDS_luc_pair-kits.pdf</t>
+  </si>
+  <si>
+    <t>Luc-Pair™ Firefly Luciferase HS Assay Kits (1000rxns)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/luc-pair-firefly-luciferase-hs-assay-kit/</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2017/02/Luc-Pair-%E2%84%A2-Firefly-Luciferase-HS-Assay-Kit-protocol.pdf</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2023/12/LF009-scaled.jpg</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2017/06/MSDS_luc_pair-kits.pdf</t>
+  </si>
+  <si>
+    <t>All-in-One™ miRNA Universal Adaptor PCR Primer (50 µM ; 20 µl)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/qpcr-mirna/#</t>
+  </si>
+  <si>
+    <t>50 µM ; 20 µl</t>
+  </si>
+  <si>
+    <t>qPCR primer</t>
+  </si>
+  <si>
+    <t>Store in –20°C and avoid repeated freeze-thaw cycles.</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2025/08/QP029-US-scaled.jpg</t>
+  </si>
+  <si>
+    <t>EndoFectin™ Lenti transfection reagent (1ml)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2015/12/EndoFectin-Lenti-Protocol.pdf</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2025/08/EF001-US-scaled.jpg</t>
+  </si>
+  <si>
+    <t>SV40 small T &amp; large T antigen Purified Lentifect™ Lentiviral Particles (25 µl x 4 vial) (old cat# LPP-SV40T-Lv105-100-C)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/product/lentiviral-particles/</t>
+  </si>
+  <si>
+    <t>eGFP-Lv105 Lentifect™ Purified Lentiviral Particles (25 µl x 1 vial)(Old cat # LPP-EGFP-Lv105-025-C)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2019/12/EGFP-Lv105-LP303-025-LP303-100.pdf</t>
+  </si>
+  <si>
+    <t>EndoFectin™ Lenti transfection reagent (3ml)</t>
+  </si>
+  <si>
+    <t>https://www.genecopoeia.com/wp-content/uploads/2025/08/EF002-US-scaled.jpg</t>
   </si>
 </sst>
 </file>
@@ -1270,443 +1474,446 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BY10"/>
+  <dimension ref="A1:BY24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>52</v>
+      </c>
+      <c r="R1" t="s">
+        <v>53</v>
+      </c>
+      <c r="S1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" t="s">
+        <v>55</v>
+      </c>
+      <c r="U1" t="s">
+        <v>56</v>
+      </c>
+      <c r="V1" t="s">
+        <v>57</v>
+      </c>
+      <c r="W1" t="s">
+        <v>58</v>
+      </c>
+      <c r="X1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AN1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M1" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O1" t="s">
-        <v>53</v>
-      </c>
-      <c r="P1" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>55</v>
-      </c>
-      <c r="R1" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" t="s">
-        <v>57</v>
-      </c>
-      <c r="T1" t="s">
-        <v>58</v>
-      </c>
-      <c r="U1" t="s">
-        <v>59</v>
-      </c>
-      <c r="V1" t="s">
-        <v>60</v>
-      </c>
-      <c r="W1" t="s">
-        <v>61</v>
-      </c>
-      <c r="X1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>14</v>
-      </c>
-      <c r="AF1" t="s">
+      <c r="AO1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AU1" t="s">
         <v>66</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AV1" t="s">
         <v>67</v>
       </c>
-      <c r="AH1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AJ1" t="s">
+      <c r="AW1" t="s">
         <v>68</v>
       </c>
-      <c r="AK1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AU1" t="s">
+      <c r="AX1" t="s">
         <v>69</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AY1" t="s">
         <v>70</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AZ1" t="s">
         <v>71</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BA1" t="s">
         <v>72</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BB1" t="s">
         <v>73</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BC1" t="s">
         <v>74</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BD1" t="s">
         <v>75</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BE1" t="s">
         <v>76</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BF1" t="s">
         <v>77</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BG1" t="s">
         <v>78</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BH1" t="s">
         <v>79</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BI1" t="s">
         <v>80</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BJ1" t="s">
         <v>81</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BK1" t="s">
         <v>82</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BL1" t="s">
         <v>83</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BM1" t="s">
         <v>84</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BN1" t="s">
         <v>85</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BO1" t="s">
         <v>86</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BP1" t="s">
         <v>87</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BQ1" t="s">
         <v>88</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BR1" t="s">
         <v>89</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BS1" t="s">
         <v>90</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BT1" t="s">
         <v>91</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BU1" t="s">
         <v>92</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BV1" t="s">
         <v>93</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BW1" t="s">
         <v>94</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BX1" t="s">
         <v>95</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BY1" t="s">
         <v>96</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>97</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>108</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB2">
-        <v>30029000</v>
-      </c>
-      <c r="AC2">
+        <v>109</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>111</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>112</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>270</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>113</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR2">
+        <v>38220090</v>
+      </c>
+      <c r="AS2">
         <v>41000000</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>28</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>132</v>
-      </c>
-      <c r="AN2" s="1">
-        <v>641</v>
       </c>
     </row>
     <row r="3" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="I3" t="s">
-        <v>35</v>
+        <v>146</v>
+      </c>
+      <c r="K3" t="s">
+        <v>147</v>
+      </c>
+      <c r="L3" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB3">
+        <v>382219</v>
+      </c>
+      <c r="AC3">
+        <v>41000000</v>
       </c>
       <c r="AD3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE3" t="s">
-        <v>34</v>
+        <v>149</v>
+      </c>
+      <c r="AF3" s="1">
+        <v>1205</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>1810</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>28</v>
       </c>
       <c r="AI3" t="s">
-        <v>37</v>
+        <v>150</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>151</v>
       </c>
       <c r="AK3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="AL3" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="AM3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AN3" s="1">
-        <v>319</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>36</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>133</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AR3">
-        <v>38220090</v>
-      </c>
-      <c r="AS3">
-        <v>41000000</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>129</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
+        <v>26</v>
+      </c>
+      <c r="K4" t="s">
+        <v>155</v>
+      </c>
+      <c r="L4" t="s">
+        <v>154</v>
+      </c>
+      <c r="AB4">
+        <v>30029000</v>
+      </c>
+      <c r="AC4">
+        <v>41000000</v>
       </c>
       <c r="AD4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE4" t="s">
-        <v>102</v>
+        <v>156</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>28</v>
       </c>
       <c r="AI4" t="s">
-        <v>103</v>
+        <v>29</v>
       </c>
       <c r="AK4" t="s">
-        <v>104</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>135</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="AN4" s="1">
-        <v>135</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AP4" t="s">
-        <v>100</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AR4">
-        <v>38220090</v>
-      </c>
-      <c r="AS4">
-        <v>41000000</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="5" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>130</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="I5" t="s">
-        <v>35</v>
+        <v>158</v>
       </c>
       <c r="AD5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE5" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="AI5" t="s">
-        <v>37</v>
+        <v>160</v>
       </c>
       <c r="AK5" t="s">
-        <v>38</v>
+        <v>161</v>
       </c>
       <c r="AL5" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="AM5" t="s">
-        <v>108</v>
+        <v>163</v>
       </c>
       <c r="AN5" s="1">
-        <v>524</v>
+        <v>410</v>
       </c>
       <c r="AO5" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="AP5" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="AQ5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="AR5">
         <v>38220090</v>
@@ -1715,54 +1922,54 @@
         <v>41000000</v>
       </c>
       <c r="AT5" t="s">
-        <v>110</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="I6" t="s">
-        <v>112</v>
+        <v>32</v>
       </c>
       <c r="AD6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE6" t="s">
-        <v>113</v>
+        <v>31</v>
       </c>
       <c r="AI6" t="s">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="AK6" t="s">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="AL6" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="AM6" t="s">
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="AN6" s="1">
-        <v>270</v>
+        <v>319</v>
       </c>
       <c r="AO6" t="s">
-        <v>116</v>
+        <v>33</v>
       </c>
       <c r="AP6" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="AQ6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="AR6">
         <v>38220090</v>
@@ -1773,99 +1980,105 @@
     </row>
     <row r="7" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>131</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="D7" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="I7" t="s">
-        <v>117</v>
-      </c>
-      <c r="K7" t="s">
-        <v>109</v>
-      </c>
-      <c r="L7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AB7">
-        <v>30029000</v>
-      </c>
-      <c r="AC7">
+        <v>158</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>161</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>163</v>
+      </c>
+      <c r="AN7" s="1">
+        <v>151</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>168</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>166</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR7">
+        <v>38220090</v>
+      </c>
+      <c r="AS7">
         <v>41000000</v>
       </c>
-      <c r="AD7" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE7" t="s">
-        <v>139</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>31</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>104</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>137</v>
-      </c>
-      <c r="AN7" s="1">
-        <v>784</v>
+      <c r="AT7" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="I8" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="AD8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE8" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="AI8" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="AK8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="AL8" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="AM8" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="AN8" s="1">
-        <v>1065</v>
+        <v>135</v>
       </c>
       <c r="AO8" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="AP8" t="s">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="AQ8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="AR8">
         <v>38220090</v>
@@ -1876,104 +2089,852 @@
     </row>
     <row r="9" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="I9" t="s">
-        <v>124</v>
+        <v>26</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB9">
+        <v>30029000</v>
+      </c>
+      <c r="AC9">
+        <v>41000000</v>
       </c>
       <c r="AD9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE9" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH9" t="s">
         <v>28</v>
       </c>
       <c r="AI9" t="s">
-        <v>125</v>
+        <v>29</v>
       </c>
       <c r="AK9" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="AL9" t="s">
-        <v>143</v>
-      </c>
-      <c r="AM9" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AN9" s="1">
-        <v>359</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>127</v>
-      </c>
-      <c r="AP9" t="s">
-        <v>142</v>
-      </c>
-      <c r="AQ9" t="s">
-        <v>31</v>
-      </c>
-      <c r="AR9">
-        <v>293499</v>
-      </c>
-      <c r="AS9">
-        <v>41000000</v>
+        <v>641</v>
       </c>
     </row>
     <row r="10" spans="1:77" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>132</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>132</v>
       </c>
       <c r="C10" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="D10" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="I10" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="AD10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE10" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="AI10" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="AK10" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="AL10" t="s">
-        <v>137</v>
+        <v>162</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>163</v>
       </c>
       <c r="AN10" s="1">
-        <v>75</v>
+        <v>432</v>
       </c>
       <c r="AO10" t="s">
-        <v>131</v>
+        <v>171</v>
       </c>
       <c r="AP10" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="AQ10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="AR10">
         <v>38220090</v>
       </c>
       <c r="AS10">
+        <v>41000000</v>
+      </c>
+      <c r="AT10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" t="s">
+        <v>172</v>
+      </c>
+      <c r="I11" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>173</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>122</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>36</v>
+      </c>
+      <c r="AN11" s="1">
+        <v>638</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>172</v>
+      </c>
+      <c r="AQ11" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR11">
+        <v>38220090</v>
+      </c>
+      <c r="AS11">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" t="s">
+        <v>174</v>
+      </c>
+      <c r="D12" t="s">
+        <v>174</v>
+      </c>
+      <c r="I12" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" t="s">
+        <v>175</v>
+      </c>
+      <c r="L12" t="s">
+        <v>174</v>
+      </c>
+      <c r="AB12">
+        <v>30029000</v>
+      </c>
+      <c r="AC12">
+        <v>41000000</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>176</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>29</v>
+      </c>
+      <c r="AK12" t="s">
+        <v>161</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>177</v>
+      </c>
+      <c r="AN12" s="1">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D13" t="s">
+        <v>178</v>
+      </c>
+      <c r="I13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>117</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>128</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN13" s="1">
+        <v>427</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>119</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>178</v>
+      </c>
+      <c r="AQ13" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR13">
+        <v>38220090</v>
+      </c>
+      <c r="AS13">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" t="s">
+        <v>180</v>
+      </c>
+      <c r="I14" t="s">
+        <v>158</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>170</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>161</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>163</v>
+      </c>
+      <c r="AN14" s="1">
+        <v>1037</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>181</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>180</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR14">
+        <v>38220090</v>
+      </c>
+      <c r="AS14">
+        <v>41000000</v>
+      </c>
+      <c r="AT14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I15" t="s">
+        <v>184</v>
+      </c>
+      <c r="J15" t="s">
+        <v>185</v>
+      </c>
+      <c r="K15" t="s">
+        <v>106</v>
+      </c>
+      <c r="L15" t="s">
+        <v>186</v>
+      </c>
+      <c r="AB15">
+        <v>30029000</v>
+      </c>
+      <c r="AC15">
+        <v>41000000</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>114</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>125</v>
+      </c>
+      <c r="AN15" s="1">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="16" spans="1:77" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B16" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D16" t="s">
+        <v>188</v>
+      </c>
+      <c r="I16" t="s">
+        <v>189</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>170</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>161</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>190</v>
+      </c>
+      <c r="AN16" s="1">
+        <v>1059</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>191</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>188</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR16">
+        <v>38220090</v>
+      </c>
+      <c r="AS16">
+        <v>41000000</v>
+      </c>
+      <c r="AT16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B17" t="s">
+        <v>138</v>
+      </c>
+      <c r="C17" t="s">
+        <v>193</v>
+      </c>
+      <c r="D17" t="s">
+        <v>193</v>
+      </c>
+      <c r="I17" t="s">
+        <v>194</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>170</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>161</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>195</v>
+      </c>
+      <c r="AN17" s="1">
+        <v>406</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>196</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>193</v>
+      </c>
+      <c r="AQ17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR17">
+        <v>38220090</v>
+      </c>
+      <c r="AS17">
+        <v>41000000</v>
+      </c>
+      <c r="AT17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>139</v>
+      </c>
+      <c r="B18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C18" t="s">
+        <v>198</v>
+      </c>
+      <c r="D18" t="s">
+        <v>198</v>
+      </c>
+      <c r="I18" t="s">
+        <v>199</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>200</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>201</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>30</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>202</v>
+      </c>
+      <c r="AN18" s="1">
+        <v>63</v>
+      </c>
+      <c r="AO18" t="s">
+        <v>203</v>
+      </c>
+      <c r="AP18" t="s">
+        <v>198</v>
+      </c>
+      <c r="AQ18" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR18">
+        <v>38220090</v>
+      </c>
+      <c r="AS18">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>116</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>117</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN19" s="1">
+        <v>1065</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>119</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AQ19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR19">
+        <v>38220090</v>
+      </c>
+      <c r="AS19">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" t="s">
+        <v>124</v>
+      </c>
+      <c r="I20" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>104</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>122</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN20" s="1">
+        <v>524</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>106</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>124</v>
+      </c>
+      <c r="AQ20" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR20">
+        <v>38220090</v>
+      </c>
+      <c r="AS20">
+        <v>41000000</v>
+      </c>
+      <c r="AT20" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>140</v>
+      </c>
+      <c r="B21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21" t="s">
+        <v>204</v>
+      </c>
+      <c r="D21" t="s">
+        <v>204</v>
+      </c>
+      <c r="I21" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>31</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>122</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>205</v>
+      </c>
+      <c r="AN21" s="1">
+        <v>265</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>206</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>204</v>
+      </c>
+      <c r="AQ21" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR21">
+        <v>38220090</v>
+      </c>
+      <c r="AS21">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>141</v>
+      </c>
+      <c r="B22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" t="s">
+        <v>207</v>
+      </c>
+      <c r="D22" t="s">
+        <v>207</v>
+      </c>
+      <c r="I22" t="s">
+        <v>208</v>
+      </c>
+      <c r="K22" t="s">
+        <v>106</v>
+      </c>
+      <c r="L22" t="s">
+        <v>186</v>
+      </c>
+      <c r="AB22">
+        <v>30029000</v>
+      </c>
+      <c r="AC22">
+        <v>41000000</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>126</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>114</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>125</v>
+      </c>
+      <c r="AN22" s="1">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="23" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" t="s">
+        <v>142</v>
+      </c>
+      <c r="C23" t="s">
+        <v>209</v>
+      </c>
+      <c r="D23" t="s">
+        <v>209</v>
+      </c>
+      <c r="I23" t="s">
+        <v>184</v>
+      </c>
+      <c r="J23" t="s">
+        <v>210</v>
+      </c>
+      <c r="K23" t="s">
+        <v>106</v>
+      </c>
+      <c r="L23" t="s">
+        <v>186</v>
+      </c>
+      <c r="AB23">
+        <v>30029000</v>
+      </c>
+      <c r="AC23">
+        <v>41000000</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>114</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>125</v>
+      </c>
+      <c r="AN23" s="1">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="24" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C24" t="s">
+        <v>211</v>
+      </c>
+      <c r="D24" t="s">
+        <v>211</v>
+      </c>
+      <c r="I24" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>173</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>122</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>205</v>
+      </c>
+      <c r="AN24" s="1">
+        <v>529</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>212</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ24" t="s">
+        <v>28</v>
+      </c>
+      <c r="AR24">
+        <v>38220090</v>
+      </c>
+      <c r="AS24">
         <v>41000000</v>
       </c>
     </row>

</xml_diff>